<commit_message>
adapt training material to removed resource relaxation step
</commit_message>
<xml_diff>
--- a/training/training_parameters.xlsx
+++ b/training/training_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\model_supply_regions\Model-Supply-Regions-MSR-Toolset\training\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/MSR code repo/training/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B07BFBB-CE56-4535-A6C2-2257093F6C78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{0B07BFBB-CE56-4535-A6C2-2257093F6C78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A05F0C1D-89C6-4B8C-AE85-941C7BD2C71D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2C5C7772-7330-4FC8-8BB5-8B002123F26F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{2C5C7772-7330-4FC8-8BB5-8B002123F26F}"/>
   </bookViews>
   <sheets>
     <sheet name="msr_creator" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
   <si>
     <t>General parameters</t>
   </si>
@@ -55,12 +55,6 @@
   </si>
   <si>
     <t>elevation_threshold</t>
-  </si>
-  <si>
-    <t>resource_relaxation_step</t>
-  </si>
-  <si>
-    <t>region_area_threshold</t>
   </si>
   <si>
     <t>land_cover_classes</t>
@@ -555,15 +549,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57FF96EB-79A6-4CAD-84E2-B265A175CC1B}">
-  <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B40"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -571,7 +565,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -579,7 +573,7 @@
         <v>2700</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -587,7 +581,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -595,84 +589,84 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>8760</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
       <c r="B9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10">
-        <v>8760</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B11">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
       <c r="B15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
       <c r="B16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -680,182 +674,166 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
       <c r="B18">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
       <c r="B19">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
       <c r="B24">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>23</v>
       </c>
       <c r="B25">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>24</v>
       </c>
       <c r="B26">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>25</v>
       </c>
-      <c r="B27">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
         <v>27</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B28" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>29</v>
       </c>
-      <c r="B30" t="s">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B31">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>32</v>
       </c>
       <c r="B33">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>33</v>
       </c>
       <c r="B34">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>34</v>
       </c>
       <c r="B35">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>35</v>
       </c>
       <c r="B36">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>36</v>
       </c>
       <c r="B37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>37</v>
       </c>
       <c r="B38">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>38</v>
       </c>
-      <c r="B39">
-        <v>1.96</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
         <v>40</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B40" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>42</v>
-      </c>
-      <c r="B42" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -866,20 +844,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9609DF47-BC50-45CA-8FEC-251AA8539B00}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B1">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -887,41 +865,41 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>8760</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>365</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>92</v>

</xml_diff>